<commit_message>
corrects column headers in sample
</commit_message>
<xml_diff>
--- a/resources/sample-meetings.xlsx
+++ b/resources/sample-meetings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/Projects/district/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/Projects/recovery/district-utils/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D663B4-C359-4942-A77E-9B90CB14DEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2559E1-7A07-A14A-B8C7-C0F2880BFC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16220" yWindow="9160" windowWidth="48980" windowHeight="27060" xr2:uid="{534B3F1F-5574-6041-84AB-D100DB8A8EBA}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t xml:space="preserve">DIST        </t>
   </si>
   <si>
-    <t xml:space="preserve">PLACE       </t>
-  </si>
-  <si>
     <t>STREET</t>
   </si>
   <si>
@@ -65,9 +62,6 @@
     <t>ZIP</t>
   </si>
   <si>
-    <t>SPECIAL INSTRUCTIONS</t>
-  </si>
-  <si>
     <t xml:space="preserve">TIME        </t>
   </si>
   <si>
@@ -77,24 +71,6 @@
     <t>MOTM</t>
   </si>
   <si>
-    <t>SEC FIRST NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-MAIL      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHONE 1     </t>
-  </si>
-  <si>
-    <t>ZoomID</t>
-  </si>
-  <si>
-    <t>ZoomPasscode</t>
-  </si>
-  <si>
-    <t>ZoomURL</t>
-  </si>
-  <si>
     <t>It's Six O'clock Somewhere (Virtual)</t>
   </si>
   <si>
@@ -279,6 +255,30 @@
   </si>
   <si>
     <t>Some Location Name</t>
+  </si>
+  <si>
+    <t>LOCATION</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>SEC_FIRST_NAME</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>PHONE</t>
+  </si>
+  <si>
+    <t>ZOOM_ID</t>
+  </si>
+  <si>
+    <t>ZOOM_PASSCODE</t>
+  </si>
+  <si>
+    <t>ZOOM_URL</t>
   </si>
 </sst>
 </file>
@@ -684,13 +684,13 @@
     <col min="10" max="10" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
@@ -704,57 +704,57 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1">
         <v>1234567</v>
@@ -763,37 +763,37 @@
         <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H2" s="1">
         <v>53201</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K2" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L2" t="s">
-        <v>44</v>
-      </c>
-      <c r="M2" s="1"/>
-      <c r="N2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="15" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1">
         <v>1234567</v>
@@ -802,16 +802,16 @@
         <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H3" s="1">
         <v>53201</v>
@@ -820,15 +820,15 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="L3" t="s">
-        <v>44</v>
-      </c>
-      <c r="N3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" ht="15" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B4" s="1">
         <v>1234567</v>
@@ -837,16 +837,16 @@
         <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H4" s="1">
         <v>53201</v>
@@ -855,16 +855,16 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L4" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="1"/>
-      <c r="N4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="15" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>65</v>
+      </c>
+      <c r="S4" s="1"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1">
         <v>1234567</v>
@@ -873,37 +873,37 @@
         <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H5" s="1">
         <v>53202</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="K5" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L5" t="s">
-        <v>38</v>
-      </c>
-      <c r="M5" s="1"/>
-      <c r="N5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="15" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="M5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S5" s="1"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B6" s="1">
         <v>1234567</v>
@@ -912,16 +912,16 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H6" s="1">
         <v>53201</v>
@@ -930,15 +930,15 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="L6" t="s">
-        <v>38</v>
-      </c>
-      <c r="N6" t="s">
-        <v>77</v>
+        <v>30</v>
+      </c>
+      <c r="M6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1">
         <v>1234567</v>
@@ -947,16 +947,16 @@
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H7" s="1">
         <v>53201</v>
@@ -965,16 +965,16 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L7" t="s">
-        <v>38</v>
-      </c>
-      <c r="M7" s="1"/>
-      <c r="N7" t="s">
-        <v>73</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="M7" t="s">
+        <v>65</v>
+      </c>
+      <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1">
         <v>1234567</v>
@@ -983,37 +983,37 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H8" s="1">
         <v>53202</v>
       </c>
       <c r="J8" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="K8" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L8" t="s">
-        <v>50</v>
-      </c>
-      <c r="M8" s="1"/>
-      <c r="N8" t="s">
-        <v>51</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="M8" t="s">
+        <v>43</v>
+      </c>
+      <c r="S8" s="1"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B9" s="1">
         <v>1234567</v>
@@ -1022,16 +1022,16 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H9" s="1">
         <v>53201</v>
@@ -1040,15 +1040,15 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="L9" t="s">
-        <v>50</v>
-      </c>
-      <c r="N9" t="s">
-        <v>77</v>
+        <v>42</v>
+      </c>
+      <c r="M9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B10" s="1">
         <v>1234567</v>
@@ -1057,16 +1057,16 @@
         <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H10" s="1">
         <v>53201</v>
@@ -1075,16 +1075,16 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L10" t="s">
-        <v>50</v>
-      </c>
-      <c r="M10" s="1"/>
-      <c r="N10" t="s">
-        <v>73</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="M10" t="s">
+        <v>65</v>
+      </c>
+      <c r="S10" s="1"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B11" s="1">
         <v>1234567</v>
@@ -1093,37 +1093,37 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H11" s="1">
         <v>53201</v>
       </c>
       <c r="J11" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="K11" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L11" t="s">
-        <v>66</v>
-      </c>
-      <c r="M11" s="1"/>
-      <c r="N11" t="s">
-        <v>67</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="M11" t="s">
+        <v>59</v>
+      </c>
+      <c r="S11" s="1"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B12" s="1">
         <v>1234567</v>
@@ -1132,37 +1132,37 @@
         <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H12" s="1">
         <v>53202</v>
       </c>
       <c r="J12" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="K12" s="2">
         <v>0.33333333333333331</v>
       </c>
       <c r="L12" t="s">
-        <v>66</v>
-      </c>
-      <c r="M12" s="1"/>
-      <c r="N12" t="s">
-        <v>71</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="M12" t="s">
+        <v>63</v>
+      </c>
+      <c r="S12" s="1"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B13" s="1">
         <v>1234567</v>
@@ -1171,37 +1171,37 @@
         <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H13" s="1">
         <v>53202</v>
       </c>
       <c r="J13" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="K13" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L13" t="s">
-        <v>62</v>
-      </c>
-      <c r="M13" s="1"/>
-      <c r="N13" t="s">
-        <v>63</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="M13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S13" s="1"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1">
         <v>1234567</v>
@@ -1210,16 +1210,16 @@
         <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H14" s="1">
         <v>53201</v>
@@ -1228,16 +1228,16 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L14" t="s">
-        <v>62</v>
-      </c>
-      <c r="M14" s="1"/>
-      <c r="N14" t="s">
-        <v>73</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="M14" t="s">
+        <v>65</v>
+      </c>
+      <c r="S14" s="1"/>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B15" s="1">
         <v>1234567</v>
@@ -1246,39 +1246,39 @@
         <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H15" s="1">
         <v>53201</v>
       </c>
       <c r="J15" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="K15" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L15" t="s">
-        <v>32</v>
-      </c>
-      <c r="M15" s="1" t="b">
+        <v>24</v>
+      </c>
+      <c r="M15" t="s">
+        <v>25</v>
+      </c>
+      <c r="S15" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="N15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B16" s="1">
         <v>1234567</v>
@@ -1287,16 +1287,16 @@
         <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H16" s="1">
         <v>53201</v>
@@ -1305,15 +1305,15 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="L16" t="s">
-        <v>32</v>
-      </c>
-      <c r="N16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="15" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+      <c r="M16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1">
         <v>1234567</v>
@@ -1322,16 +1322,16 @@
         <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F17" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H17" s="1">
         <v>53201</v>
@@ -1340,15 +1340,15 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="15" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+      <c r="M17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B18" s="1">
         <v>1234567</v>
@@ -1357,37 +1357,37 @@
         <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F18" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H18" s="1">
         <v>53201</v>
       </c>
       <c r="J18" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="K18" s="2">
         <v>0.70833333333333337</v>
       </c>
       <c r="L18" t="s">
-        <v>56</v>
-      </c>
-      <c r="M18" s="1"/>
-      <c r="N18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="15" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="M18" t="s">
+        <v>49</v>
+      </c>
+      <c r="S18" s="1"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B19" s="1">
         <v>1234567</v>
@@ -1396,16 +1396,16 @@
         <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H19" s="1">
         <v>53201</v>
@@ -1414,15 +1414,15 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="L19" t="s">
-        <v>56</v>
-      </c>
-      <c r="N19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="15" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="M19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B20" s="1">
         <v>1234567</v>
@@ -1431,16 +1431,16 @@
         <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H20" s="1">
         <v>53201</v>
@@ -1449,16 +1449,16 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="L20" t="s">
-        <v>56</v>
-      </c>
-      <c r="M20" s="1"/>
-      <c r="N20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" ht="15" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="M20" t="s">
+        <v>65</v>
+      </c>
+      <c r="S20" s="1"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B21" s="1">
         <v>1234567</v>
@@ -1467,32 +1467,32 @@
         <v>38</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2">
         <v>0.75</v>
       </c>
       <c r="L21" t="s">
-        <v>21</v>
-      </c>
-      <c r="M21" s="1"/>
-      <c r="N21" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q21" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="R21" t="s">
-        <v>74</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="M21" t="s">
+        <v>14</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>66</v>
+      </c>
+      <c r="S21" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S22">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R22">
     <sortCondition descending="1" ref="L2:L22"/>
     <sortCondition descending="1" ref="K2:K22"/>
   </sortState>

</xml_diff>